<commit_message>
feat: support 33-node Simulink realtime data integration
</commit_message>
<xml_diff>
--- a/backend/safety/scenario.xlsx
+++ b/backend/safety/scenario.xlsx
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">

</xml_diff>